<commit_message>
Fix loi khi cap nhat Tuyen duong - ok
</commit_message>
<xml_diff>
--- a/data/giao_thong_data_upadate.xlsx
+++ b/data/giao_thong_data_upadate.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B59EFE30-1BAF-41F7-94E4-FC8737339091}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" tabRatio="959" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" tabRatio="959" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TuyenDuong" sheetId="1" r:id="rId1"/>
@@ -2974,491 +2974,6 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
         <sz val="14"/>
         <color auto="1"/>
         <name val="Arial"/>
@@ -4861,71 +4376,6 @@
       </border>
     </dxf>
     <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -5610,6 +5060,556 @@
         <bottom/>
       </border>
     </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -5624,129 +5624,129 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{55F27C45-874E-4B7C-B5FC-C409B116FDE9}" name="Table6" displayName="Table6" ref="A1:O50" totalsRowShown="0" headerRowDxfId="91" dataDxfId="89" headerRowBorderDxfId="90" tableBorderDxfId="88" totalsRowBorderDxfId="87">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{55F27C45-874E-4B7C-B5FC-C409B116FDE9}" name="Table6" displayName="Table6" ref="A1:O50" totalsRowShown="0" headerRowDxfId="72" dataDxfId="70" headerRowBorderDxfId="71" tableBorderDxfId="69" totalsRowBorderDxfId="68">
   <autoFilter ref="A1:O50" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{F7F05447-A2ED-4BD4-8A55-03ABCA25E4EA}" name="Mã tuyến" dataDxfId="86"/>
-    <tableColumn id="2" xr3:uid="{229801F1-DCEE-451E-917F-F560EA35554F}" name="Tên tuyến" dataDxfId="85"/>
-    <tableColumn id="3" xr3:uid="{4F852BC1-DBA8-4B5F-AAE2-85EC787967C2}" name="Cấp quản lý" dataDxfId="84"/>
-    <tableColumn id="4" xr3:uid="{0643DAF9-9B8D-4F87-8677-F08927D38A41}" name="CD quản lý (km)" dataDxfId="83"/>
-    <tableColumn id="5" xr3:uid="{E3B9262B-13B8-400A-B66F-BC5E9051B155}" name="CD thực tế (km)" dataDxfId="82"/>
-    <tableColumn id="6" xr3:uid="{4A72A890-C463-476A-A36A-E73D28D0ED28}" name="Đơn vị quản lý" dataDxfId="81"/>
-    <tableColumn id="7" xr3:uid="{B9E1A61C-5530-4E83-9ABD-4205A08EB961}" name="Điểm đầu" dataDxfId="80"/>
-    <tableColumn id="8" xr3:uid="{7799C677-9093-4406-8DCC-229636D13681}" name="Điểm cuối" dataDxfId="79"/>
-    <tableColumn id="9" xr3:uid="{61ABE95B-C97A-4E6B-81D5-D3A9D917D524}" name="Lat đầu" dataDxfId="78"/>
-    <tableColumn id="10" xr3:uid="{80A9BBEC-E09B-4C41-B12B-0EED1C6E387D}" name="Lng đầu" dataDxfId="77"/>
-    <tableColumn id="11" xr3:uid="{6BC6E265-AC68-4EFA-A3F5-C51F9FCD4630}" name="Lat cuối" dataDxfId="76"/>
-    <tableColumn id="12" xr3:uid="{0394693D-75DE-4B3C-B355-55CC046D98A0}" name="Lng cuối" dataDxfId="75"/>
-    <tableColumn id="13" xr3:uid="{12ACCC8A-59BC-4373-9360-E34BF0B42649}" name="Năm xây dựng" dataDxfId="74"/>
-    <tableColumn id="14" xr3:uid="{D0950277-BB12-4EA5-B75D-C1BFC3F41689}" name="Năm hoàn thành" dataDxfId="73"/>
-    <tableColumn id="15" xr3:uid="{3D449CF7-2B8B-430A-A3E6-2C3924E85C05}" name="Ghi chú" dataDxfId="72"/>
+    <tableColumn id="1" xr3:uid="{F7F05447-A2ED-4BD4-8A55-03ABCA25E4EA}" name="Mã tuyến" dataDxfId="67"/>
+    <tableColumn id="2" xr3:uid="{229801F1-DCEE-451E-917F-F560EA35554F}" name="Tên tuyến" dataDxfId="66"/>
+    <tableColumn id="3" xr3:uid="{4F852BC1-DBA8-4B5F-AAE2-85EC787967C2}" name="Cấp quản lý" dataDxfId="65"/>
+    <tableColumn id="4" xr3:uid="{0643DAF9-9B8D-4F87-8677-F08927D38A41}" name="CD quản lý (km)" dataDxfId="64"/>
+    <tableColumn id="5" xr3:uid="{E3B9262B-13B8-400A-B66F-BC5E9051B155}" name="CD thực tế (km)" dataDxfId="63"/>
+    <tableColumn id="6" xr3:uid="{4A72A890-C463-476A-A36A-E73D28D0ED28}" name="Đơn vị quản lý" dataDxfId="62"/>
+    <tableColumn id="7" xr3:uid="{B9E1A61C-5530-4E83-9ABD-4205A08EB961}" name="Điểm đầu" dataDxfId="61"/>
+    <tableColumn id="8" xr3:uid="{7799C677-9093-4406-8DCC-229636D13681}" name="Điểm cuối" dataDxfId="60"/>
+    <tableColumn id="9" xr3:uid="{61ABE95B-C97A-4E6B-81D5-D3A9D917D524}" name="Lat đầu" dataDxfId="59"/>
+    <tableColumn id="10" xr3:uid="{80A9BBEC-E09B-4C41-B12B-0EED1C6E387D}" name="Lng đầu" dataDxfId="58"/>
+    <tableColumn id="11" xr3:uid="{6BC6E265-AC68-4EFA-A3F5-C51F9FCD4630}" name="Lat cuối" dataDxfId="57"/>
+    <tableColumn id="12" xr3:uid="{0394693D-75DE-4B3C-B355-55CC046D98A0}" name="Lng cuối" dataDxfId="56"/>
+    <tableColumn id="13" xr3:uid="{12ACCC8A-59BC-4373-9360-E34BF0B42649}" name="Năm xây dựng" dataDxfId="55"/>
+    <tableColumn id="14" xr3:uid="{D0950277-BB12-4EA5-B75D-C1BFC3F41689}" name="Năm hoàn thành" dataDxfId="54"/>
+    <tableColumn id="15" xr3:uid="{3D449CF7-2B8B-430A-A3E6-2C3924E85C05}" name="Ghi chú" dataDxfId="53"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B72143DA-3681-41AD-900A-B1B168684B34}" name="Table1" displayName="Table1" ref="A1:N223" totalsRowShown="0" headerRowDxfId="71" dataDxfId="0" headerRowBorderDxfId="70" tableBorderDxfId="69" totalsRowBorderDxfId="68">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B72143DA-3681-41AD-900A-B1B168684B34}" name="Table1" displayName="Table1" ref="A1:N223" totalsRowShown="0" headerRowDxfId="91" dataDxfId="89" headerRowBorderDxfId="90" tableBorderDxfId="88" totalsRowBorderDxfId="87">
   <autoFilter ref="A1:N223" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{5A243110-AA3F-4506-BE0B-E61914F44435}" name="Mã đoạn" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{82748143-6448-4AC1-9B61-3287A1A950D2}" name="Mã tuyến" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{A6D8BCE3-DA6C-4708-980E-0EAC148F3127}" name="Cấp đường" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{7F4805D2-6F33-434B-88EA-A61738A6C9B7}" name="Lý trình đầu (km)" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{BC7E5F0A-83EB-4E90-A5BF-DA91EDDA20A7}" name="Lý trình cuối (km)" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{94F84141-9DB5-4566-B3B6-FA657E4B1490}" name="Tình trạng" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{72850592-D43B-41CB-AD16-319982C5F1D9}" name="Chiều dài thực tế (km)" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{0238CC43-94BA-4344-9F14-9ADE7AA5AAC5}" name="Mã kết cấu mặt" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{7E65411B-1444-4D30-8135-555A0D8A0023}" name="Rộng mặt min (m)" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{44E4AF34-9504-4DD0-A38B-406A83C5B104}" name="Rộng mặt max (m)" dataDxfId="5"/>
-    <tableColumn id="11" xr3:uid="{54D13739-A782-4FB1-9CA7-ABF900E5DC7B}" name="Rộng nền min (m)" dataDxfId="4"/>
-    <tableColumn id="12" xr3:uid="{33053654-9134-4F85-B95C-EAA7B2AEFBB2}" name="Rộng nền max (m)" dataDxfId="3"/>
-    <tableColumn id="13" xr3:uid="{177149AC-EA8E-4C96-B7A8-0537E1885222}" name="Đơn vị bảo dưỡng" dataDxfId="2"/>
-    <tableColumn id="14" xr3:uid="{CC78A5BB-8A19-42EE-984E-305B0B5EDFED}" name="Ghi chú" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{5A243110-AA3F-4506-BE0B-E61914F44435}" name="Mã đoạn" dataDxfId="86"/>
+    <tableColumn id="2" xr3:uid="{82748143-6448-4AC1-9B61-3287A1A950D2}" name="Mã tuyến" dataDxfId="85"/>
+    <tableColumn id="3" xr3:uid="{A6D8BCE3-DA6C-4708-980E-0EAC148F3127}" name="Cấp đường" dataDxfId="84"/>
+    <tableColumn id="4" xr3:uid="{7F4805D2-6F33-434B-88EA-A61738A6C9B7}" name="Lý trình đầu (km)" dataDxfId="83"/>
+    <tableColumn id="5" xr3:uid="{BC7E5F0A-83EB-4E90-A5BF-DA91EDDA20A7}" name="Lý trình cuối (km)" dataDxfId="82"/>
+    <tableColumn id="6" xr3:uid="{94F84141-9DB5-4566-B3B6-FA657E4B1490}" name="Tình trạng" dataDxfId="81"/>
+    <tableColumn id="7" xr3:uid="{72850592-D43B-41CB-AD16-319982C5F1D9}" name="Chiều dài thực tế (km)" dataDxfId="80"/>
+    <tableColumn id="8" xr3:uid="{0238CC43-94BA-4344-9F14-9ADE7AA5AAC5}" name="Mã kết cấu mặt" dataDxfId="79"/>
+    <tableColumn id="9" xr3:uid="{7E65411B-1444-4D30-8135-555A0D8A0023}" name="Rộng mặt min (m)" dataDxfId="78"/>
+    <tableColumn id="10" xr3:uid="{44E4AF34-9504-4DD0-A38B-406A83C5B104}" name="Rộng mặt max (m)" dataDxfId="77"/>
+    <tableColumn id="11" xr3:uid="{54D13739-A782-4FB1-9CA7-ABF900E5DC7B}" name="Rộng nền min (m)" dataDxfId="76"/>
+    <tableColumn id="12" xr3:uid="{33053654-9134-4F85-B95C-EAA7B2AEFBB2}" name="Rộng nền max (m)" dataDxfId="75"/>
+    <tableColumn id="13" xr3:uid="{177149AC-EA8E-4C96-B7A8-0537E1885222}" name="Đơn vị bảo dưỡng" dataDxfId="74"/>
+    <tableColumn id="14" xr3:uid="{CC78A5BB-8A19-42EE-984E-305B0B5EDFED}" name="Ghi chú" dataDxfId="73"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{21743309-9187-4405-B529-43F40707C652}" name="Table18" displayName="Table18" ref="A1:I16" totalsRowShown="0" headerRowDxfId="67" dataDxfId="65" headerRowBorderDxfId="66" tableBorderDxfId="64" totalsRowBorderDxfId="63">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{21743309-9187-4405-B529-43F40707C652}" name="Table18" displayName="Table18" ref="A1:I16" totalsRowShown="0" headerRowDxfId="52" dataDxfId="50" headerRowBorderDxfId="51" tableBorderDxfId="49" totalsRowBorderDxfId="48">
   <autoFilter ref="A1:I16" xr:uid="{21743309-9187-4405-B529-43F40707C652}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{62DDD64A-B2E2-4AC3-9378-0BEAD395D5D6}" name="Tuyến đi chung" dataDxfId="62"/>
-    <tableColumn id="11" xr3:uid="{39C1441E-E76E-497B-8A84-9E7CFC21FDE8}" name="Tuyến chính" dataDxfId="61"/>
-    <tableColumn id="2" xr3:uid="{B088B7D5-DB99-4940-B18F-254EDD0FBBAA}" name="Mã đoạn (tuyến chủ)" dataDxfId="60"/>
-    <tableColumn id="3" xr3:uid="{8F0B5946-C9F0-45D2-9765-910A823F14A0}" name="Lý trình đầu đi chung" dataDxfId="59"/>
-    <tableColumn id="4" xr3:uid="{DA635A7C-93E9-4B79-90FB-E73EA17433D2}" name="Lý trình cuối đi chung" dataDxfId="58"/>
-    <tableColumn id="6" xr3:uid="{36A160D8-4911-428B-BC35-6F7150A50625}" name="Lý trình đầu tuyến chính" dataDxfId="57"/>
-    <tableColumn id="7" xr3:uid="{EF3B275C-85DF-4502-85FF-1DFDB0DD3822}" name="Lý trình cuối tuyến chính" dataDxfId="56"/>
-    <tableColumn id="12" xr3:uid="{B5D35CF0-B366-4ECE-80C0-822A413B8134}" name="Chiều dài đoạn đi chung" dataDxfId="55"/>
-    <tableColumn id="5" xr3:uid="{DA66B68B-1302-4273-AF51-CBCB691AA306}" name="Ghi chú" dataDxfId="54"/>
+    <tableColumn id="1" xr3:uid="{62DDD64A-B2E2-4AC3-9378-0BEAD395D5D6}" name="Tuyến đi chung" dataDxfId="47"/>
+    <tableColumn id="11" xr3:uid="{39C1441E-E76E-497B-8A84-9E7CFC21FDE8}" name="Tuyến chính" dataDxfId="46"/>
+    <tableColumn id="2" xr3:uid="{B088B7D5-DB99-4940-B18F-254EDD0FBBAA}" name="Mã đoạn (tuyến chủ)" dataDxfId="45"/>
+    <tableColumn id="3" xr3:uid="{8F0B5946-C9F0-45D2-9765-910A823F14A0}" name="Lý trình đầu đi chung" dataDxfId="44"/>
+    <tableColumn id="4" xr3:uid="{DA635A7C-93E9-4B79-90FB-E73EA17433D2}" name="Lý trình cuối đi chung" dataDxfId="43"/>
+    <tableColumn id="6" xr3:uid="{36A160D8-4911-428B-BC35-6F7150A50625}" name="Lý trình đầu tuyến chính" dataDxfId="42"/>
+    <tableColumn id="7" xr3:uid="{EF3B275C-85DF-4502-85FF-1DFDB0DD3822}" name="Lý trình cuối tuyến chính" dataDxfId="41"/>
+    <tableColumn id="12" xr3:uid="{B5D35CF0-B366-4ECE-80C0-822A413B8134}" name="Chiều dài đoạn đi chung" dataDxfId="40"/>
+    <tableColumn id="5" xr3:uid="{DA66B68B-1302-4273-AF51-CBCB691AA306}" name="Ghi chú" dataDxfId="39"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{407DEAA1-417A-4B24-8FAC-755EDDFB46F2}" name="Table2" displayName="Table2" ref="A1:C10" totalsRowShown="0" headerRowDxfId="53" headerRowBorderDxfId="52" tableBorderDxfId="51" totalsRowBorderDxfId="50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{407DEAA1-417A-4B24-8FAC-755EDDFB46F2}" name="Table2" displayName="Table2" ref="A1:C10" totalsRowShown="0" headerRowDxfId="38" headerRowBorderDxfId="37" tableBorderDxfId="36" totalsRowBorderDxfId="35">
   <autoFilter ref="A1:C10" xr:uid="{407DEAA1-417A-4B24-8FAC-755EDDFB46F2}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{A3FFD2B3-91E7-4EB2-85C8-BB4468C9A928}" name="ma" dataDxfId="49"/>
-    <tableColumn id="2" xr3:uid="{5C404D1F-878C-4C02-9910-27C755DCEF79}" name="ten" dataDxfId="48"/>
-    <tableColumn id="3" xr3:uid="{3401E260-BFBE-4F45-8103-87B9F81A238B}" name="mo_ta" dataDxfId="47"/>
+    <tableColumn id="1" xr3:uid="{A3FFD2B3-91E7-4EB2-85C8-BB4468C9A928}" name="ma" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{5C404D1F-878C-4C02-9910-27C755DCEF79}" name="ten" dataDxfId="33"/>
+    <tableColumn id="3" xr3:uid="{3401E260-BFBE-4F45-8103-87B9F81A238B}" name="mo_ta" dataDxfId="32"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{4BA7F0B0-CDB5-4FDA-A663-3910215DD203}" name="Table3" displayName="Table3" ref="A1:D18" totalsRowShown="0" headerRowDxfId="46" headerRowBorderDxfId="45" tableBorderDxfId="44" totalsRowBorderDxfId="43">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{4BA7F0B0-CDB5-4FDA-A663-3910215DD203}" name="Table3" displayName="Table3" ref="A1:D18" totalsRowShown="0" headerRowDxfId="31" headerRowBorderDxfId="30" tableBorderDxfId="29" totalsRowBorderDxfId="28">
   <autoFilter ref="A1:D18" xr:uid="{4BA7F0B0-CDB5-4FDA-A663-3910215DD203}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{5E8E435D-A5D0-446A-8F6C-15CFB008990B}" name="Mã đơn vị" dataDxfId="42"/>
-    <tableColumn id="2" xr3:uid="{7A962071-338A-4D61-8380-4218224837F9}" name="Tên đơn vị" dataDxfId="41"/>
-    <tableColumn id="3" xr3:uid="{A9E300B8-9A70-40C7-8295-F211A6DFDDC5}" name="Loại đơn vị" dataDxfId="40"/>
-    <tableColumn id="4" xr3:uid="{0F2F093E-9010-4E3F-9A1E-4D374646A1BE}" name="parent_id" dataDxfId="39"/>
+    <tableColumn id="1" xr3:uid="{5E8E435D-A5D0-446A-8F6C-15CFB008990B}" name="Mã đơn vị" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{7A962071-338A-4D61-8380-4218224837F9}" name="Tên đơn vị" dataDxfId="26"/>
+    <tableColumn id="3" xr3:uid="{A9E300B8-9A70-40C7-8295-F211A6DFDDC5}" name="Loại đơn vị" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{0F2F093E-9010-4E3F-9A1E-4D374646A1BE}" name="parent_id" dataDxfId="24"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{449D73CD-396F-4A94-BF28-46F00E104F59}" name="Table4" displayName="Table4" ref="A1:D9" totalsRowShown="0" headerRowDxfId="38" headerRowBorderDxfId="37" tableBorderDxfId="36" totalsRowBorderDxfId="35">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{449D73CD-396F-4A94-BF28-46F00E104F59}" name="Table4" displayName="Table4" ref="A1:D9" totalsRowShown="0" headerRowDxfId="23" headerRowBorderDxfId="22" tableBorderDxfId="21" totalsRowBorderDxfId="20">
   <autoFilter ref="A1:D9" xr:uid="{449D73CD-396F-4A94-BF28-46F00E104F59}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{7DAF5E0B-9E0F-44EB-A68E-23C9B90C6C58}" name="ma_cap" dataDxfId="34"/>
-    <tableColumn id="2" xr3:uid="{1BD33F16-36D8-4E2A-80E6-7C8A655AA250}" name="ten_cap" dataDxfId="33"/>
-    <tableColumn id="3" xr3:uid="{A9EE3611-21E9-488F-87A9-55E28BD30330}" name="mo_ta" dataDxfId="32"/>
-    <tableColumn id="4" xr3:uid="{9BFD356E-605B-400A-898F-E405602E418F}" name="thu_tu_hien_thi" dataDxfId="31"/>
+    <tableColumn id="1" xr3:uid="{7DAF5E0B-9E0F-44EB-A68E-23C9B90C6C58}" name="ma_cap" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{1BD33F16-36D8-4E2A-80E6-7C8A655AA250}" name="ten_cap" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{A9EE3611-21E9-488F-87A9-55E28BD30330}" name="mo_ta" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{9BFD356E-605B-400A-898F-E405602E418F}" name="thu_tu_hien_thi" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{90A226A7-C9D1-4372-B503-85C7C1814ADA}" name="Table11" displayName="Table11" ref="A1:D8" totalsRowShown="0" headerRowDxfId="30" dataDxfId="29" tableBorderDxfId="28">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{90A226A7-C9D1-4372-B503-85C7C1814ADA}" name="Table11" displayName="Table11" ref="A1:D8" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14" tableBorderDxfId="13">
   <autoFilter ref="A1:D8" xr:uid="{90A226A7-C9D1-4372-B503-85C7C1814ADA}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{F753712D-BD5B-42DE-B7E4-8F3D0D176E28}" name="Ma_cap" dataDxfId="27"/>
-    <tableColumn id="2" xr3:uid="{5B0101BE-0DC0-4393-B522-B6F65F4F604A}" name="ten_cap" dataDxfId="26"/>
-    <tableColumn id="3" xr3:uid="{B2AFA268-16FC-4B91-A4DB-C3B6AB9776BA}" name="mo_ta" dataDxfId="25"/>
-    <tableColumn id="4" xr3:uid="{68E65E67-2F35-400E-B704-91E4FBB614F6}" name="thu_tu_hien_thi" dataDxfId="24"/>
+    <tableColumn id="1" xr3:uid="{F753712D-BD5B-42DE-B7E4-8F3D0D176E28}" name="Ma_cap" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{5B0101BE-0DC0-4393-B522-B6F65F4F604A}" name="ten_cap" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{B2AFA268-16FC-4B91-A4DB-C3B6AB9776BA}" name="mo_ta" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{68E65E67-2F35-400E-B704-91E4FBB614F6}" name="thu_tu_hien_thi" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{92BB339D-7159-42AA-905D-C393F6AFD807}" name="Table510" displayName="Table510" ref="A1:D9" totalsRowShown="0" headerRowDxfId="23" dataDxfId="21" headerRowBorderDxfId="22" tableBorderDxfId="20" totalsRowBorderDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{92BB339D-7159-42AA-905D-C393F6AFD807}" name="Table510" displayName="Table510" ref="A1:D9" totalsRowShown="0" headerRowDxfId="8" dataDxfId="6" headerRowBorderDxfId="7" tableBorderDxfId="5" totalsRowBorderDxfId="4">
   <autoFilter ref="A1:D9" xr:uid="{92BB339D-7159-42AA-905D-C393F6AFD807}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{30F91324-8313-456E-85EA-0A930AEE777F}" name="ma_ket_cau" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{BB9B7B6D-9381-42A7-B1FB-A44D4A5ED483}" name="ten_ket_cau" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{5C1BE301-15D1-401C-BDE8-6603435072FC}" name="mo_ta" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{771FD841-AD7F-4F26-B6FE-38DE31EF9426}" name="thu_tu_hien_thi" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{30F91324-8313-456E-85EA-0A930AEE777F}" name="ma_ket_cau" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{BB9B7B6D-9381-42A7-B1FB-A44D4A5ED483}" name="ten_ket_cau" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{5C1BE301-15D1-401C-BDE8-6603435072FC}" name="mo_ta" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{771FD841-AD7F-4F26-B6FE-38DE31EF9426}" name="thu_tu_hien_thi" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>